<commit_message>
v1.0.0: add version management, remove legacy validation-rule-map config
- add ban-ben-guan-li/VERSION_MANIFEST.json, CHANGELOG.md, README.md
- add PyCode/core/app_identity.py: single source for product name/version,
  works in both source tree and frozen exe
- menu banner now shows 'pytools V1.0.0'
- build_exe.bat: build from spec, name artifact 'pytools V{ver}_{timestamp}.exe',
  keep previous exe on build failure
- specs bundle VERSION_MANIFEST.json as data
- remove obsolete 'jiao-yan-gui-ze-ying-she-biao' sheet, dead loader and
  maintenance code; config repair now purges the legacy sheet automatically
</commit_message>
<xml_diff>
--- a/PyCode/config/config.xlsx
+++ b/PyCode/config/config.xlsx
@@ -18,11 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="归档类型配置" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交检查配置" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件排序配置" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="校验规则映射表" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'校验规则映射表'!$A$1:$J$4</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -369,66 +366,6 @@
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>备注字段（仅人工说明）：程序不读取。</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>pytools</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：Y/是/1/true 表示启用该映射行。</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：必须与校验关系工作簿中的Sheet名称完全一致，例如 表8-1。</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：该组映射对应的报表口径，例如 D、F、J。</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：报表年份标识，例如 26；同Sheet、同口径、同年份组成一组映射。</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：关系式中的表格名称，例如 表8-1；同表关系未写表名时默认使用校验关系Sheet。</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：正式报表编码，不含行列部分，例如 S0801_J_26。</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：指标前缀取自指标名称开头，例如 1、1.1、2；按完整前缀精确匹配。</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>关键字段（程序读取）：指标在正式报表中的实际行编号，例如 1；输出时自动补为001。</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>可选字段：关系式未写.A/.B等列编号时使用；关系式已写列编号时以关系式为准。</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>备注字段（仅人工说明）：程序不读取，可填写指标名称便于维护。</t>
       </text>
     </comment>
   </commentList>
@@ -1803,242 +1740,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>是否启用</t>
-        </is>
-      </c>
-      <c r="B1" s="12" t="inlineStr">
-        <is>
-          <t>校验关系Sheet</t>
-        </is>
-      </c>
-      <c r="C1" s="12" t="inlineStr">
-        <is>
-          <t>口径</t>
-        </is>
-      </c>
-      <c r="D1" s="12" t="inlineStr">
-        <is>
-          <t>年份</t>
-        </is>
-      </c>
-      <c r="E1" s="12" t="inlineStr">
-        <is>
-          <t>表格名称</t>
-        </is>
-      </c>
-      <c r="F1" s="12" t="inlineStr">
-        <is>
-          <t>表格编码</t>
-        </is>
-      </c>
-      <c r="G1" s="12" t="inlineStr">
-        <is>
-          <t>指标前缀</t>
-        </is>
-      </c>
-      <c r="H1" s="12" t="inlineStr">
-        <is>
-          <t>实际行编号</t>
-        </is>
-      </c>
-      <c r="I1" s="12" t="inlineStr">
-        <is>
-          <t>默认列编号</t>
-        </is>
-      </c>
-      <c r="J1" s="12" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>表8-1</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>表8-1</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>S0801_J_26</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" s="13" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>资产</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>表8-1</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>表8-1</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>S0801_J_26</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>资产子项1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>表8-1</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>表8-1</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>S0801_J_26</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>003</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>资产子项2</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:J4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>